<commit_message>
T4: embed chart images (render in Excel for Mac) alongside native charts
Add make_charts.py (reproducible PNGs) and embed the rendered images at the
top of T4_EVs_chart and T4_elec_chart, so the 3-scenario charts display even
when Excel for Mac does not render native openpyxl charts. Native charts kept
below the images. Electricity mix shows all 3 scenarios (CDN/SNBC/LTS).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ssp_modeling/cost-benefits/crosswalk/morocco_crosswalk_deliverable.xlsx
+++ b/ssp_modeling/cost-benefits/crosswalk/morocco_crosswalk_deliverable.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="374">
   <si>
     <t xml:space="preserve">Morocco investment &amp; benefits crosswalk</t>
   </si>
@@ -780,6 +780,9 @@
     <t xml:space="preserve">Stacked area of the ESTIMATION blocks in T4_vehicles (vehicles = VKM / divisor). Reproduces the Tableau 'EVs-Private' (road_light) and 'EVs-Public' (public, road_heavy_freight) views. Note under LTS: road_light -&gt; Electricity, road_heavy_freight -&gt; Hydrogen.</t>
   </si>
   <si>
+    <t xml:space="preserve">Rendered images (guaranteed to display); interactive native charts are further below.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Private light vehicles (road_light, /12,000)</t>
   </si>
   <si>
@@ -868,6 +871,9 @@
   </si>
   <si>
     <t xml:space="preserve">Stacked area of the SHARE-OF-TOTAL blocks in T4_elec_generation. Reproduces the Tableau 'Electricity Generation by Source Morocco'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendered image (guaranteed to display); interactive native charts are further below.</t>
   </si>
   <si>
     <t xml:space="preserve">Task 4 — Total final energy demand by fuel (LEDS)</t>
@@ -2642,11 +2648,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="7003496"/>
-        <c:axId val="18393866"/>
+        <c:axId val="4476191"/>
+        <c:axId val="76547763"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="7003496"/>
+        <c:axId val="4476191"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2712,7 +2718,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18393866"/>
+        <c:crossAx val="76547763"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2720,7 +2726,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18393866"/>
+        <c:axId val="76547763"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2796,7 +2802,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7003496"/>
+        <c:crossAx val="4476191"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -5323,11 +5329,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="96268537"/>
-        <c:axId val="2759035"/>
+        <c:axId val="83818073"/>
+        <c:axId val="57457701"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="96268537"/>
+        <c:axId val="83818073"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5393,7 +5399,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2759035"/>
+        <c:crossAx val="57457701"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5401,7 +5407,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2759035"/>
+        <c:axId val="57457701"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5477,7 +5483,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96268537"/>
+        <c:crossAx val="83818073"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -8004,11 +8010,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="5869303"/>
-        <c:axId val="17957734"/>
+        <c:axId val="83065921"/>
+        <c:axId val="14230107"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="5869303"/>
+        <c:axId val="83065921"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8074,7 +8080,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17957734"/>
+        <c:crossAx val="14230107"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8082,7 +8088,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="17957734"/>
+        <c:axId val="14230107"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8158,7 +8164,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5869303"/>
+        <c:crossAx val="83065921"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -10685,11 +10691,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="68832843"/>
-        <c:axId val="24227941"/>
+        <c:axId val="54036295"/>
+        <c:axId val="3291891"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="68832843"/>
+        <c:axId val="54036295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10755,7 +10761,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24227941"/>
+        <c:crossAx val="3291891"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -10763,7 +10769,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24227941"/>
+        <c:axId val="3291891"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -10839,7 +10845,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68832843"/>
+        <c:crossAx val="54036295"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -11908,11 +11914,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="32029309"/>
-        <c:axId val="1237608"/>
+        <c:axId val="42283758"/>
+        <c:axId val="85901902"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="32029309"/>
+        <c:axId val="42283758"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -11978,7 +11984,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1237608"/>
+        <c:crossAx val="85901902"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -11986,7 +11992,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1237608"/>
+        <c:axId val="85901902"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -12062,7 +12068,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32029309"/>
+        <c:crossAx val="42283758"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -13131,11 +13137,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="26368307"/>
-        <c:axId val="77378583"/>
+        <c:axId val="5255668"/>
+        <c:axId val="38115295"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="26368307"/>
+        <c:axId val="5255668"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13201,7 +13207,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77378583"/>
+        <c:crossAx val="38115295"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -13209,7 +13215,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77378583"/>
+        <c:axId val="38115295"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -13285,7 +13291,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26368307"/>
+        <c:crossAx val="5255668"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -14111,11 +14117,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="67140832"/>
-        <c:axId val="12274507"/>
+        <c:axId val="45480972"/>
+        <c:axId val="95058541"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="67140832"/>
+        <c:axId val="45480972"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14181,7 +14187,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12274507"/>
+        <c:crossAx val="95058541"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -14189,7 +14195,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="12274507"/>
+        <c:axId val="95058541"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -14265,7 +14271,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67140832"/>
+        <c:crossAx val="45480972"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -15091,11 +15097,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="60230097"/>
-        <c:axId val="90918849"/>
+        <c:axId val="2129923"/>
+        <c:axId val="18189968"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="60230097"/>
+        <c:axId val="2129923"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15161,7 +15167,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90918849"/>
+        <c:crossAx val="18189968"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -15169,7 +15175,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90918849"/>
+        <c:axId val="18189968"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -15245,7 +15251,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60230097"/>
+        <c:crossAx val="2129923"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -16071,11 +16077,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="81885408"/>
-        <c:axId val="16264291"/>
+        <c:axId val="16632426"/>
+        <c:axId val="68628803"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="81885408"/>
+        <c:axId val="16632426"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16141,7 +16147,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16264291"/>
+        <c:crossAx val="68628803"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -16149,7 +16155,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="16264291"/>
+        <c:axId val="68628803"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -16225,7 +16231,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81885408"/>
+        <c:crossAx val="16632426"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -17537,11 +17543,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="53312744"/>
-        <c:axId val="53944637"/>
+        <c:axId val="64531417"/>
+        <c:axId val="39957600"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="53312744"/>
+        <c:axId val="64531417"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17607,7 +17613,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53944637"/>
+        <c:crossAx val="39957600"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -17615,7 +17621,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="53944637"/>
+        <c:axId val="39957600"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -17691,7 +17697,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53312744"/>
+        <c:crossAx val="64531417"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -19003,11 +19009,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="12443200"/>
-        <c:axId val="78690320"/>
+        <c:axId val="99199155"/>
+        <c:axId val="59373723"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="12443200"/>
+        <c:axId val="99199155"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -19073,7 +19079,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78690320"/>
+        <c:crossAx val="59373723"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -19081,7 +19087,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78690320"/>
+        <c:axId val="59373723"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -19157,7 +19163,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12443200"/>
+        <c:crossAx val="99199155"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -20469,11 +20475,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="18330644"/>
-        <c:axId val="48930293"/>
+        <c:axId val="34435706"/>
+        <c:axId val="23938139"/>
       </c:areaChart>
       <c:catAx>
-        <c:axId val="18330644"/>
+        <c:axId val="34435706"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -20539,7 +20545,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48930293"/>
+        <c:crossAx val="23938139"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -20547,7 +20553,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48930293"/>
+        <c:axId val="23938139"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -20623,7 +20629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18330644"/>
+        <c:crossAx val="34435706"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -23276,14 +23282,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>56</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23291,7 +23297,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="762120"/>
+        <a:off x="0" y="10667880"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23306,14 +23312,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>73</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23321,7 +23327,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="4000680"/>
+        <a:off x="0" y="13906440"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23336,13 +23342,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>90</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>53</xdr:row>
+      <xdr:row>105</xdr:row>
       <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -23351,7 +23357,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="7238880"/>
+        <a:off x="0" y="17145000"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23366,14 +23372,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>110</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23381,7 +23387,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="11049120"/>
+        <a:off x="0" y="20954880"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23396,14 +23402,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>75</xdr:row>
+      <xdr:row>127</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>90</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23411,7 +23417,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="14287680"/>
+        <a:off x="0" y="24193440"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23426,13 +23432,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>144</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>107</xdr:row>
+      <xdr:row>159</xdr:row>
       <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -23441,7 +23447,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="17525880"/>
+        <a:off x="0" y="27432000"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23456,14 +23462,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>112</xdr:row>
+      <xdr:row>164</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>127</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23471,7 +23477,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="21336120"/>
+        <a:off x="0" y="31241880"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23486,14 +23492,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>129</xdr:row>
+      <xdr:row>181</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>144</xdr:row>
-      <xdr:rowOff>22320</xdr:rowOff>
+      <xdr:row>196</xdr:row>
+      <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -23501,7 +23507,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="24574680"/>
+        <a:off x="0" y="34480440"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23516,13 +23522,13 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>146</xdr:row>
+      <xdr:row>198</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>473040</xdr:colOff>
-      <xdr:row>161</xdr:row>
+      <xdr:row>213</xdr:row>
       <xdr:rowOff>21960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
@@ -23531,7 +23537,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="27812880"/>
+        <a:off x="0" y="37719000"/>
         <a:ext cx="7199640" cy="2879640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23540,6 +23546,82 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>352080</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>28440</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Image 10" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId10"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="9524520" cy="3076200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>352080</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>75960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Image 11" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId11"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="5143680"/>
+          <a:ext cx="9524520" cy="5409720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -23551,22 +23633,22 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>78480</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>1440</xdr:rowOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="10" name="Chart 1"/>
+        <xdr:cNvPr id="12" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="571680"/>
+        <a:off x="0" y="5524560"/>
         <a:ext cx="8639640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23581,22 +23663,22 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>48</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>78480</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>65</xdr:row>
       <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="11" name="Chart 2"/>
+        <xdr:cNvPr id="13" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="4191120"/>
+        <a:off x="0" y="9144000"/>
         <a:ext cx="8639640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23611,22 +23693,22 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
+      <xdr:row>67</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>78480</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>84</xdr:row>
       <xdr:rowOff>1080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="12" name="Chart 3"/>
+        <xdr:cNvPr id="14" name="Chart 3"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="7810560"/>
+        <a:off x="0" y="12763440"/>
         <a:ext cx="8639640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -23635,6 +23717,44 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>81360</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>133200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="762120"/>
+          <a:ext cx="10477080" cy="3752640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -37597,7 +37717,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A112"/>
+  <dimension ref="A1:A164"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37611,18 +37731,23 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="23" t="s">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="23" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="23" t="s">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="23" t="s">
         <v>249</v>
+      </c>
+    </row>
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="23" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -37650,47 +37775,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -37709,34 +37834,34 @@
         <v>113</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>58</v>
@@ -38836,7 +38961,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B41" s="12"/>
       <c r="C41" s="12"/>
@@ -38855,34 +38980,34 @@
         <v>113</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I42" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L42" s="3" t="s">
         <v>58</v>
@@ -39982,7 +40107,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B72" s="12"/>
       <c r="C72" s="12"/>
@@ -40001,34 +40126,34 @@
         <v>113</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I73" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K73" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L73" s="3" t="s">
         <v>58</v>
@@ -41128,12 +41253,12 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B105" s="12"/>
       <c r="C105" s="12"/>
@@ -41151,34 +41276,34 @@
         <v>113</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E106" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K106" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -42443,7 +42568,7 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B137" s="12"/>
       <c r="C137" s="12"/>
@@ -42461,34 +42586,34 @@
         <v>113</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F138" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I138" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J138" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K138" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43753,7 +43878,7 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="10" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B169" s="12"/>
       <c r="C169" s="12"/>
@@ -43771,34 +43896,34 @@
         <v>113</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E170" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G170" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="H170" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="I170" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="J170" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="K170" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45077,17 +45202,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>276</v>
+        <v>277</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="22" t="s">
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -45116,12 +45246,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45129,79 +45259,79 @@
         <v>113</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="Y3" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="Z3" s="3" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -47871,36 +48001,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B6" s="30" t="n">
         <v>372</v>
@@ -47916,7 +48046,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B7" s="30" t="n">
         <v>339</v>
@@ -47932,7 +48062,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B8" s="30" t="n">
         <v>862</v>
@@ -47948,7 +48078,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B9" s="30" t="n">
         <v>990</v>
@@ -47964,7 +48094,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B10" s="10" t="n">
         <f aca="false">SUM(B6:B9)</f>
@@ -47978,44 +48108,44 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B13" s="33" t="n">
         <v>299</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B14" s="33" t="n">
         <v>152</v>
       </c>
       <c r="C14" s="34" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="35" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48023,12 +48153,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
   </sheetData>
@@ -48055,7 +48185,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48063,47 +48193,47 @@
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48111,62 +48241,62 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
   </sheetData>
@@ -48197,17 +48327,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="36" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48215,19 +48345,19 @@
         <v>169</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48244,10 +48374,10 @@
         <v>384.893</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48264,10 +48394,10 @@
         <v>167.066</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F7" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48284,10 +48414,10 @@
         <v>64.759</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48304,10 +48434,10 @@
         <v>39.991</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F9" s="38" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48324,10 +48454,10 @@
         <v>32.758</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F10" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48344,10 +48474,10 @@
         <v>32.59</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48364,10 +48494,10 @@
         <v>25.855</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F12" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48384,15 +48514,15 @@
         <v>25.694</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>0</v>
@@ -48404,10 +48534,10 @@
         <v>17.427</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F14" s="38" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48424,10 +48554,10 @@
         <v>12.106</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48444,15 +48574,15 @@
         <v>-3.867</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B17" s="7" t="n">
         <v>0</v>
@@ -48464,15 +48594,15 @@
         <v>8.135</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F17" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>0</v>
@@ -48484,10 +48614,10 @@
         <v>4.795</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F18" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48504,15 +48634,15 @@
         <v>3.193</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F19" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>0</v>
@@ -48524,10 +48654,10 @@
         <v>0.047</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F20" s="38" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48544,45 +48674,45 @@
         <v>-3.401</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="35" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -48590,12 +48720,12 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>